<commit_message>
Added 2022 soil analysis and fixed ObjectId case errors
</commit_message>
<xml_diff>
--- a/Data/2022_F013B4_CO_ISSWC/2022_F013B4_CO_ISSWC_CropCanopy.xlsx
+++ b/Data/2022_F013B4_CO_ISSWC/2022_F013B4_CO_ISSWC_CropCanopy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2022_F013B4_CO_ISSWC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F77BDA4B-81C9-43CD-A879-CB1F59256DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9014B42F-0135-4C6E-976E-FEFA8BBE69EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16470" yWindow="-19380" windowWidth="17805" windowHeight="18345" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16470" yWindow="-19380" windowWidth="17805" windowHeight="18345" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Height" sheetId="9" r:id="rId1"/>
@@ -53139,14 +53139,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECA672C-8ED2-4A38-91F5-3D50AA22177A}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="118" t="s">
         <v>227</v>
       </c>
@@ -53163,9 +53164,8 @@
         <v>231</v>
       </c>
       <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-    </row>
-    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="119" t="s">
         <v>210</v>
       </c>
@@ -53178,11 +53178,11 @@
       <c r="D2" s="304">
         <v>124.25</v>
       </c>
-      <c r="E2" s="304">
-        <v>134.125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E2" s="303">
+        <v>44695</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="119" t="s">
         <v>207</v>
       </c>
@@ -53195,11 +53195,11 @@
       <c r="D3" s="304">
         <v>122.5</v>
       </c>
-      <c r="E3" s="304">
-        <v>133.75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E3" s="303">
+        <v>44695</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="119" t="s">
         <v>204</v>
       </c>
@@ -53212,11 +53212,11 @@
       <c r="D4" s="304">
         <v>124.1</v>
       </c>
-      <c r="E4" s="304">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E4" s="303">
+        <v>44696</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="119" t="s">
         <v>201</v>
       </c>
@@ -53229,11 +53229,11 @@
       <c r="D5" s="304">
         <v>123</v>
       </c>
-      <c r="E5" s="304">
-        <v>133.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E5" s="303">
+        <v>44695</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="119" t="s">
         <v>198</v>
       </c>
@@ -53246,11 +53246,11 @@
       <c r="D6" s="304">
         <v>121.25</v>
       </c>
-      <c r="E6" s="304">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E6" s="303">
+        <v>44693</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="119" t="s">
         <v>195</v>
       </c>
@@ -53263,11 +53263,11 @@
       <c r="D7" s="304">
         <v>121</v>
       </c>
-      <c r="E7" s="304">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E7" s="303">
+        <v>44694</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="119" t="s">
         <v>192</v>
       </c>
@@ -53280,11 +53280,11 @@
       <c r="D8" s="304">
         <v>120.5</v>
       </c>
-      <c r="E8" s="304">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E8" s="303">
+        <v>44692</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="119" t="s">
         <v>189</v>
       </c>
@@ -53297,11 +53297,11 @@
       <c r="D9" s="304">
         <v>120.8</v>
       </c>
-      <c r="E9" s="304">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E9" s="303">
+        <v>44693</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="119" t="s">
         <v>186</v>
       </c>
@@ -53314,11 +53314,11 @@
       <c r="D10" s="304">
         <v>124.25</v>
       </c>
-      <c r="E10" s="304">
-        <v>134.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E10" s="303">
+        <v>44696</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="119" t="s">
         <v>183</v>
       </c>
@@ -53331,11 +53331,11 @@
       <c r="D11" s="304">
         <v>121.35714285714286</v>
       </c>
-      <c r="E11" s="304">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E11" s="303">
+        <v>44695</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="119" t="s">
         <v>180</v>
       </c>
@@ -53348,11 +53348,11 @@
       <c r="D12" s="304">
         <v>120.8</v>
       </c>
-      <c r="E12" s="304">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E12" s="303">
+        <v>44695</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="119" t="s">
         <v>177</v>
       </c>
@@ -53365,11 +53365,11 @@
       <c r="D13" s="304">
         <v>124.125</v>
       </c>
-      <c r="E13" s="304">
-        <v>135.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E13" s="303">
+        <v>44697</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="119" t="s">
         <v>174</v>
       </c>
@@ -53382,11 +53382,11 @@
       <c r="D14" s="304">
         <v>120.8</v>
       </c>
-      <c r="E14" s="304">
-        <v>132.25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E14" s="303">
+        <v>44693</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="119" t="s">
         <v>171</v>
       </c>
@@ -53399,11 +53399,11 @@
       <c r="D15" s="304">
         <v>121.25</v>
       </c>
-      <c r="E15" s="304">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="E15" s="303">
+        <v>44694</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="119" t="s">
         <v>168</v>
       </c>
@@ -53416,8 +53416,8 @@
       <c r="D16" s="304">
         <v>122.16666666666667</v>
       </c>
-      <c r="E16" s="304">
-        <v>133.5</v>
+      <c r="E16" s="303">
+        <v>44695</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53433,8 +53433,8 @@
       <c r="D17" s="304">
         <v>120.5</v>
       </c>
-      <c r="E17" s="304">
-        <v>132.5</v>
+      <c r="E17" s="303">
+        <v>44694</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53450,8 +53450,8 @@
       <c r="D18" s="304">
         <v>121.1</v>
       </c>
-      <c r="E18" s="304">
-        <v>133.375</v>
+      <c r="E18" s="303">
+        <v>44694</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53467,8 +53467,8 @@
       <c r="D19" s="304">
         <v>121.25</v>
       </c>
-      <c r="E19" s="304">
-        <v>132.5</v>
+      <c r="E19" s="303">
+        <v>44694</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53484,8 +53484,8 @@
       <c r="D20" s="304">
         <v>122</v>
       </c>
-      <c r="E20" s="304">
-        <v>132.25</v>
+      <c r="E20" s="303">
+        <v>44693</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53501,8 +53501,8 @@
       <c r="D21" s="304">
         <v>120.5</v>
       </c>
-      <c r="E21" s="304">
-        <v>133.375</v>
+      <c r="E21" s="303">
+        <v>44694</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53518,8 +53518,8 @@
       <c r="D22" s="304">
         <v>121.1</v>
       </c>
-      <c r="E22" s="304">
-        <v>134.5</v>
+      <c r="E22" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53535,8 +53535,8 @@
       <c r="D23" s="304">
         <v>123.5</v>
       </c>
-      <c r="E23" s="304">
-        <v>136.5</v>
+      <c r="E23" s="303">
+        <v>44698</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53552,8 +53552,8 @@
       <c r="D24" s="304">
         <v>122.5</v>
       </c>
-      <c r="E24" s="304">
-        <v>134.5</v>
+      <c r="E24" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53569,8 +53569,8 @@
       <c r="D25" s="304">
         <v>125</v>
       </c>
-      <c r="E25" s="304">
-        <v>136.75</v>
+      <c r="E25" s="303">
+        <v>44698</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53586,8 +53586,8 @@
       <c r="D26" s="304">
         <v>122.25</v>
       </c>
-      <c r="E26" s="304">
-        <v>133.75</v>
+      <c r="E26" s="303">
+        <v>44695</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53603,8 +53603,8 @@
       <c r="D27" s="304">
         <v>122</v>
       </c>
-      <c r="E27" s="304">
-        <v>133</v>
+      <c r="E27" s="303">
+        <v>44694</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53620,8 +53620,8 @@
       <c r="D28" s="304">
         <v>120.75</v>
       </c>
-      <c r="E28" s="304">
-        <v>131.875</v>
+      <c r="E28" s="303">
+        <v>44693</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53637,8 +53637,8 @@
       <c r="D29" s="304">
         <v>121.625</v>
       </c>
-      <c r="E29" s="304">
-        <v>134.5</v>
+      <c r="E29" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53654,8 +53654,8 @@
       <c r="D30" s="304">
         <v>124.25</v>
       </c>
-      <c r="E30" s="304">
-        <v>135.25</v>
+      <c r="E30" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53671,8 +53671,8 @@
       <c r="D31" s="304">
         <v>122.75</v>
       </c>
-      <c r="E31" s="304">
-        <v>134.5</v>
+      <c r="E31" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53688,8 +53688,8 @@
       <c r="D32" s="304">
         <v>122.25</v>
       </c>
-      <c r="E32" s="304">
-        <v>134.875</v>
+      <c r="E32" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53705,8 +53705,8 @@
       <c r="D33" s="304">
         <v>123</v>
       </c>
-      <c r="E33" s="304">
-        <v>136.75</v>
+      <c r="E33" s="303">
+        <v>44698</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53722,8 +53722,8 @@
       <c r="D34" s="304">
         <v>125</v>
       </c>
-      <c r="E34" s="304">
-        <v>136</v>
+      <c r="E34" s="303">
+        <v>44697</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53739,8 +53739,8 @@
       <c r="D35" s="304">
         <v>122.83333333333333</v>
       </c>
-      <c r="E35" s="304">
-        <v>134.5</v>
+      <c r="E35" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53756,8 +53756,8 @@
       <c r="D36" s="304">
         <v>125.8</v>
       </c>
-      <c r="E36" s="304">
-        <v>135.25</v>
+      <c r="E36" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53773,8 +53773,8 @@
       <c r="D37" s="304">
         <v>122.25</v>
       </c>
-      <c r="E37" s="304">
-        <v>137.16666666666666</v>
+      <c r="E37" s="303">
+        <v>44698</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53790,8 +53790,8 @@
       <c r="D38" s="304">
         <v>122</v>
       </c>
-      <c r="E38" s="304">
-        <v>134</v>
+      <c r="E38" s="303">
+        <v>44695</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53807,8 +53807,8 @@
       <c r="D39" s="304">
         <v>121.625</v>
       </c>
-      <c r="E39" s="304">
-        <v>135.5</v>
+      <c r="E39" s="303">
+        <v>44697</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53824,8 +53824,8 @@
       <c r="D40" s="304">
         <v>122.3</v>
       </c>
-      <c r="E40" s="304">
-        <v>133.5</v>
+      <c r="E40" s="303">
+        <v>44695</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53841,8 +53841,8 @@
       <c r="D41" s="304">
         <v>121</v>
       </c>
-      <c r="E41" s="304">
-        <v>133</v>
+      <c r="E41" s="303">
+        <v>44694</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53858,8 +53858,8 @@
       <c r="D42" s="304">
         <v>122</v>
       </c>
-      <c r="E42" s="304">
-        <v>132</v>
+      <c r="E42" s="303">
+        <v>44693</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53875,8 +53875,8 @@
       <c r="D43" s="304">
         <v>121.5</v>
       </c>
-      <c r="E43" s="304">
-        <v>134.5</v>
+      <c r="E43" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53892,8 +53892,8 @@
       <c r="D44" s="304">
         <v>121.25</v>
       </c>
-      <c r="E44" s="304">
-        <v>132.4</v>
+      <c r="E44" s="303">
+        <v>44693</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53909,8 +53909,8 @@
       <c r="D45" s="304">
         <v>121.625</v>
       </c>
-      <c r="E45" s="304">
-        <v>133.75</v>
+      <c r="E45" s="303">
+        <v>44695</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53926,8 +53926,8 @@
       <c r="D46" s="304">
         <v>125.4</v>
       </c>
-      <c r="E46" s="304">
-        <v>134.5</v>
+      <c r="E46" s="303">
+        <v>44696</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53943,8 +53943,8 @@
       <c r="D47" s="304">
         <v>123</v>
       </c>
-      <c r="E47" s="304">
-        <v>137.4</v>
+      <c r="E47" s="303">
+        <v>44698</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53960,8 +53960,8 @@
       <c r="D48" s="304">
         <v>127</v>
       </c>
-      <c r="E48" s="304">
-        <v>144.5</v>
+      <c r="E48" s="303">
+        <v>44706</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -53977,12 +53977,12 @@
       <c r="D49" s="304">
         <v>122.75</v>
       </c>
-      <c r="E49" s="304">
-        <v>139.5</v>
+      <c r="E49" s="303">
+        <v>44701</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E49">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D49">
     <sortCondition ref="A2:A49"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -53996,7 +53996,8 @@
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="13" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -54054,8 +54055,8 @@
       <c r="D2" s="304">
         <v>124.25</v>
       </c>
-      <c r="E2" s="304">
-        <v>134.125</v>
+      <c r="E2" s="303">
+        <v>44695</v>
       </c>
       <c r="F2" s="302">
         <v>8.5</v>
@@ -54095,8 +54096,8 @@
       <c r="D3" s="304">
         <v>122.5</v>
       </c>
-      <c r="E3" s="304">
-        <v>133.75</v>
+      <c r="E3" s="303">
+        <v>44695</v>
       </c>
       <c r="F3" s="302">
         <v>7.333333333333333</v>
@@ -54136,8 +54137,8 @@
       <c r="D4" s="304">
         <v>124.1</v>
       </c>
-      <c r="E4" s="304">
-        <v>135</v>
+      <c r="E4" s="303">
+        <v>44696</v>
       </c>
       <c r="F4" s="302">
         <v>8</v>
@@ -54177,8 +54178,8 @@
       <c r="D5" s="304">
         <v>123</v>
       </c>
-      <c r="E5" s="304">
-        <v>133.75</v>
+      <c r="E5" s="303">
+        <v>44695</v>
       </c>
       <c r="F5" s="302">
         <v>8.3333333333333339</v>
@@ -54218,8 +54219,8 @@
       <c r="D6" s="304">
         <v>121.25</v>
       </c>
-      <c r="E6" s="304">
-        <v>132</v>
+      <c r="E6" s="303">
+        <v>44693</v>
       </c>
       <c r="F6" s="302">
         <v>8.6666666666666661</v>
@@ -54259,8 +54260,8 @@
       <c r="D7" s="304">
         <v>121</v>
       </c>
-      <c r="E7" s="304">
-        <v>133</v>
+      <c r="E7" s="303">
+        <v>44694</v>
       </c>
       <c r="F7" s="302">
         <v>8.2222222222222214</v>
@@ -54300,8 +54301,8 @@
       <c r="D8" s="304">
         <v>120.5</v>
       </c>
-      <c r="E8" s="304">
-        <v>131</v>
+      <c r="E8" s="303">
+        <v>44692</v>
       </c>
       <c r="F8" s="302">
         <v>8.4444444444444446</v>
@@ -54341,8 +54342,8 @@
       <c r="D9" s="304">
         <v>120.8</v>
       </c>
-      <c r="E9" s="304">
-        <v>132</v>
+      <c r="E9" s="303">
+        <v>44693</v>
       </c>
       <c r="F9" s="302">
         <v>7.333333333333333</v>
@@ -54382,8 +54383,8 @@
       <c r="D10" s="304">
         <v>124.25</v>
       </c>
-      <c r="E10" s="304">
-        <v>134.5</v>
+      <c r="E10" s="303">
+        <v>44696</v>
       </c>
       <c r="F10" s="302">
         <v>7.7777777777777777</v>
@@ -54423,8 +54424,8 @@
       <c r="D11" s="304">
         <v>121.35714285714286</v>
       </c>
-      <c r="E11" s="304">
-        <v>134</v>
+      <c r="E11" s="303">
+        <v>44695</v>
       </c>
       <c r="F11" s="302">
         <v>8.4444444444444446</v>
@@ -54464,8 +54465,8 @@
       <c r="D12" s="304">
         <v>120.8</v>
       </c>
-      <c r="E12" s="304">
-        <v>134</v>
+      <c r="E12" s="303">
+        <v>44695</v>
       </c>
       <c r="F12" s="302">
         <v>8.7777777777777786</v>
@@ -54505,8 +54506,8 @@
       <c r="D13" s="304">
         <v>124.125</v>
       </c>
-      <c r="E13" s="304">
-        <v>135.5</v>
+      <c r="E13" s="303">
+        <v>44697</v>
       </c>
       <c r="F13" s="302">
         <v>8.8888888888888893</v>
@@ -54546,8 +54547,8 @@
       <c r="D14" s="304">
         <v>120.8</v>
       </c>
-      <c r="E14" s="304">
-        <v>132.25</v>
+      <c r="E14" s="303">
+        <v>44693</v>
       </c>
       <c r="F14" s="302">
         <v>8.4444444444444446</v>
@@ -54587,8 +54588,8 @@
       <c r="D15" s="304">
         <v>121.25</v>
       </c>
-      <c r="E15" s="304">
-        <v>133</v>
+      <c r="E15" s="303">
+        <v>44694</v>
       </c>
       <c r="F15" s="302">
         <v>9.3333333333333339</v>
@@ -54628,8 +54629,8 @@
       <c r="D16" s="304">
         <v>122.16666666666667</v>
       </c>
-      <c r="E16" s="304">
-        <v>133.5</v>
+      <c r="E16" s="303">
+        <v>44695</v>
       </c>
       <c r="F16" s="302">
         <v>9.5555555555555554</v>
@@ -54669,8 +54670,8 @@
       <c r="D17" s="304">
         <v>120.5</v>
       </c>
-      <c r="E17" s="304">
-        <v>132.5</v>
+      <c r="E17" s="303">
+        <v>44694</v>
       </c>
       <c r="F17" s="302">
         <v>8.4444444444444446</v>
@@ -54710,8 +54711,8 @@
       <c r="D18" s="304">
         <v>121.1</v>
       </c>
-      <c r="E18" s="304">
-        <v>133.375</v>
+      <c r="E18" s="303">
+        <v>44694</v>
       </c>
       <c r="F18" s="302">
         <v>7.4444444444444446</v>
@@ -54751,8 +54752,8 @@
       <c r="D19" s="304">
         <v>121.25</v>
       </c>
-      <c r="E19" s="304">
-        <v>132.5</v>
+      <c r="E19" s="303">
+        <v>44694</v>
       </c>
       <c r="F19" s="302">
         <v>7.8888888888888893</v>
@@ -54792,8 +54793,8 @@
       <c r="D20" s="304">
         <v>122</v>
       </c>
-      <c r="E20" s="304">
-        <v>132.25</v>
+      <c r="E20" s="303">
+        <v>44693</v>
       </c>
       <c r="F20" s="302">
         <v>7.666666666666667</v>
@@ -54833,8 +54834,8 @@
       <c r="D21" s="304">
         <v>120.5</v>
       </c>
-      <c r="E21" s="304">
-        <v>133.375</v>
+      <c r="E21" s="303">
+        <v>44694</v>
       </c>
       <c r="F21" s="302">
         <v>7.5555555555555554</v>
@@ -54874,8 +54875,8 @@
       <c r="D22" s="304">
         <v>121.1</v>
       </c>
-      <c r="E22" s="304">
-        <v>134.5</v>
+      <c r="E22" s="303">
+        <v>44696</v>
       </c>
       <c r="F22" s="302">
         <v>8.7777777777777786</v>
@@ -54915,8 +54916,8 @@
       <c r="D23" s="304">
         <v>123.5</v>
       </c>
-      <c r="E23" s="304">
-        <v>136.5</v>
+      <c r="E23" s="303">
+        <v>44698</v>
       </c>
       <c r="F23" s="302">
         <v>7.4444444444444446</v>
@@ -54956,8 +54957,8 @@
       <c r="D24" s="304">
         <v>122.5</v>
       </c>
-      <c r="E24" s="304">
-        <v>134.5</v>
+      <c r="E24" s="303">
+        <v>44696</v>
       </c>
       <c r="F24" s="302">
         <v>8.1111111111111107</v>
@@ -54997,8 +54998,8 @@
       <c r="D25" s="304">
         <v>125</v>
       </c>
-      <c r="E25" s="304">
-        <v>136.75</v>
+      <c r="E25" s="303">
+        <v>44698</v>
       </c>
       <c r="F25" s="302">
         <v>8</v>
@@ -55038,8 +55039,8 @@
       <c r="D26" s="304">
         <v>122.25</v>
       </c>
-      <c r="E26" s="304">
-        <v>133.75</v>
+      <c r="E26" s="303">
+        <v>44695</v>
       </c>
       <c r="F26" s="302">
         <v>6.4444444444444446</v>
@@ -55079,8 +55080,8 @@
       <c r="D27" s="304">
         <v>122</v>
       </c>
-      <c r="E27" s="304">
-        <v>133</v>
+      <c r="E27" s="303">
+        <v>44694</v>
       </c>
       <c r="F27" s="302">
         <v>7.5555555555555554</v>
@@ -55120,8 +55121,8 @@
       <c r="D28" s="304">
         <v>120.75</v>
       </c>
-      <c r="E28" s="304">
-        <v>131.875</v>
+      <c r="E28" s="303">
+        <v>44693</v>
       </c>
       <c r="F28" s="302">
         <v>8.3333333333333339</v>
@@ -55161,8 +55162,8 @@
       <c r="D29" s="304">
         <v>121.625</v>
       </c>
-      <c r="E29" s="304">
-        <v>134.5</v>
+      <c r="E29" s="303">
+        <v>44696</v>
       </c>
       <c r="F29" s="302">
         <v>8.3333333333333339</v>
@@ -55202,8 +55203,8 @@
       <c r="D30" s="304">
         <v>124.25</v>
       </c>
-      <c r="E30" s="304">
-        <v>135.25</v>
+      <c r="E30" s="303">
+        <v>44696</v>
       </c>
       <c r="F30" s="302">
         <v>7.1111111111111107</v>
@@ -55243,8 +55244,8 @@
       <c r="D31" s="304">
         <v>122.75</v>
       </c>
-      <c r="E31" s="304">
-        <v>134.5</v>
+      <c r="E31" s="303">
+        <v>44696</v>
       </c>
       <c r="F31" s="302">
         <v>9.1111111111111107</v>
@@ -55284,8 +55285,8 @@
       <c r="D32" s="304">
         <v>122.25</v>
       </c>
-      <c r="E32" s="304">
-        <v>134.875</v>
+      <c r="E32" s="303">
+        <v>44696</v>
       </c>
       <c r="F32" s="302">
         <v>9.2222222222222214</v>
@@ -55325,8 +55326,8 @@
       <c r="D33" s="304">
         <v>123</v>
       </c>
-      <c r="E33" s="304">
-        <v>136.75</v>
+      <c r="E33" s="303">
+        <v>44698</v>
       </c>
       <c r="F33" s="302">
         <v>8.7777777777777786</v>
@@ -55366,8 +55367,8 @@
       <c r="D34" s="304">
         <v>125</v>
       </c>
-      <c r="E34" s="304">
-        <v>136</v>
+      <c r="E34" s="303">
+        <v>44697</v>
       </c>
       <c r="F34" s="302">
         <v>8.1111111111111107</v>
@@ -55407,8 +55408,8 @@
       <c r="D35" s="304">
         <v>122.83333333333333</v>
       </c>
-      <c r="E35" s="304">
-        <v>134.5</v>
+      <c r="E35" s="303">
+        <v>44696</v>
       </c>
       <c r="F35" s="302">
         <v>8.7777777777777786</v>
@@ -55448,8 +55449,8 @@
       <c r="D36" s="304">
         <v>125.8</v>
       </c>
-      <c r="E36" s="304">
-        <v>135.25</v>
+      <c r="E36" s="303">
+        <v>44696</v>
       </c>
       <c r="F36" s="302">
         <v>8.2222222222222214</v>
@@ -55489,8 +55490,8 @@
       <c r="D37" s="304">
         <v>122.25</v>
       </c>
-      <c r="E37" s="304">
-        <v>137.16666666666666</v>
+      <c r="E37" s="303">
+        <v>44698</v>
       </c>
       <c r="F37" s="302">
         <v>8</v>
@@ -55530,8 +55531,8 @@
       <c r="D38" s="304">
         <v>122</v>
       </c>
-      <c r="E38" s="304">
-        <v>134</v>
+      <c r="E38" s="303">
+        <v>44695</v>
       </c>
       <c r="F38" s="302">
         <v>8.1111111111111107</v>
@@ -55571,8 +55572,8 @@
       <c r="D39" s="304">
         <v>121.625</v>
       </c>
-      <c r="E39" s="304">
-        <v>135.5</v>
+      <c r="E39" s="303">
+        <v>44697</v>
       </c>
       <c r="F39" s="302">
         <v>8.2222222222222214</v>
@@ -55612,8 +55613,8 @@
       <c r="D40" s="304">
         <v>122.3</v>
       </c>
-      <c r="E40" s="304">
-        <v>133.5</v>
+      <c r="E40" s="303">
+        <v>44695</v>
       </c>
       <c r="F40" s="302">
         <v>7.4444444444444446</v>
@@ -55653,8 +55654,8 @@
       <c r="D41" s="304">
         <v>121</v>
       </c>
-      <c r="E41" s="304">
-        <v>133</v>
+      <c r="E41" s="303">
+        <v>44694</v>
       </c>
       <c r="F41" s="302">
         <v>7</v>
@@ -55694,8 +55695,8 @@
       <c r="D42" s="304">
         <v>122</v>
       </c>
-      <c r="E42" s="304">
-        <v>132</v>
+      <c r="E42" s="303">
+        <v>44693</v>
       </c>
       <c r="F42" s="302">
         <v>8.1111111111111107</v>
@@ -55735,8 +55736,8 @@
       <c r="D43" s="304">
         <v>121.5</v>
       </c>
-      <c r="E43" s="304">
-        <v>134.5</v>
+      <c r="E43" s="303">
+        <v>44696</v>
       </c>
       <c r="F43" s="302">
         <v>8.4444444444444446</v>
@@ -55776,8 +55777,8 @@
       <c r="D44" s="304">
         <v>121.25</v>
       </c>
-      <c r="E44" s="304">
-        <v>132.4</v>
+      <c r="E44" s="303">
+        <v>44693</v>
       </c>
       <c r="F44" s="302">
         <v>8.5555555555555554</v>
@@ -55817,8 +55818,8 @@
       <c r="D45" s="304">
         <v>121.625</v>
       </c>
-      <c r="E45" s="304">
-        <v>133.75</v>
+      <c r="E45" s="303">
+        <v>44695</v>
       </c>
       <c r="F45" s="302">
         <v>7.4444444444444446</v>
@@ -55858,8 +55859,8 @@
       <c r="D46" s="304">
         <v>125.4</v>
       </c>
-      <c r="E46" s="304">
-        <v>134.5</v>
+      <c r="E46" s="303">
+        <v>44696</v>
       </c>
       <c r="F46" s="302">
         <v>7.2222222222222223</v>
@@ -55899,8 +55900,8 @@
       <c r="D47" s="304">
         <v>123</v>
       </c>
-      <c r="E47" s="304">
-        <v>137.4</v>
+      <c r="E47" s="303">
+        <v>44698</v>
       </c>
       <c r="F47" s="302">
         <v>8.6666666666666661</v>
@@ -55940,8 +55941,8 @@
       <c r="D48" s="304">
         <v>127</v>
       </c>
-      <c r="E48" s="304">
-        <v>144.5</v>
+      <c r="E48" s="303">
+        <v>44706</v>
       </c>
       <c r="F48" s="302">
         <v>9.3333333333333339</v>
@@ -55981,8 +55982,8 @@
       <c r="D49" s="304">
         <v>122.75</v>
       </c>
-      <c r="E49" s="304">
-        <v>139.5</v>
+      <c r="E49" s="303">
+        <v>44701</v>
       </c>
       <c r="F49" s="302">
         <v>8.3333333333333339</v>

</xml_diff>